<commit_message>
Agrega guía de Corfo, plan de la Ley 21.719 y hojas de seguimiento
- docs/corfo: guía hecha con las bases técnicas oficiales de Semilla Inicia (requisitos, cómo
  calza KeyServ, evaluación, qué falta), borrador de postulación con guion del video de 40 s y
  puente de la tesis a los documentos nuevos.
- docs/cumplimiento/PLAN_ADECUACION_LEY_21719.md: cuenta regresiva al 1-dic-2026, estado por
  área, tratamientos nuevos, plan de 6 semanas y preguntas para el abogado.
- El consentimiento del video de verificación guarda la versión del texto aceptado
  (migración 0043).
- Libro de seguimiento: hojas Corfo y Gantt, 13 tareas nuevas; changelog, índice y estado al día.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -17,14 +17,17 @@
     <sheet name="Comision" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Presupuesto" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Pruebas" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Corfo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gantt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tareas'!$A$1:$J$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cambios'!$A$1:$E$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tareas'!$A$1:$J$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cambios'!$A$1:$E$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Decisiones'!$A$1:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Pendientes_dueño'!$A$1:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Riesgos'!$A$1:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Pruebas'!$A$1:$H$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Corfo'!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,9 +35,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;[Red]-#,##0;-"/>
+    <numFmt numFmtId="166" formatCode="&quot;M&quot;0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -121,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -161,11 +165,17 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -184,6 +194,13 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="00FFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="002E75B6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -619,7 +636,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Tareas · Planner · Cambios · Decisiones · Pendientes_dueño · Riesgos · Comision (calculadora con fórmulas) · Presupuesto · Pruebas</t>
+          <t>Tareas · Planner · Cambios · Decisiones · Pendientes_dueño · Riesgos · Comision (calculadora con fórmulas) · Presupuesto · Pruebas · Corfo (requisitos de las bases) · Gantt (10 meses de ejecución)</t>
         </is>
       </c>
     </row>
@@ -1522,13 +1539,1396 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Requisito</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Acción</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Postulante</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Persona natural mayor de 18 años y residente en Chile</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.1 a)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Elegir al beneficiario entre los tres autores</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Postulante</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>No tener participación en una sociedad que ya ejecute el proyecto</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.1 a)</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>No constituir la sociedad antes de postular</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Postulante</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>No figurar en el Registro Nacional de Deudores de Pensiones de Alimentos</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Bases 9.1, 13.3</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Cada integrante lo revisa</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Postulante</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Sin otro proyecto Corfo vigente (más de 2 meses de terminar) ni cofinanciamiento previo del mismo emprendimiento</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.4</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Confirmar con cada integrante</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Postulante</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Una sola postulación por persona natural en cada convocatoria</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.4.2</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Postular una vez</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Innovación suficiente frente a las soluciones existentes</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Bases 2.1, 13.1</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Estudio de competencia chilena y propuesta de valor</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Alcance no exclusivamente local (comunal o provincial no es admisible)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Bases 2.1 c)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Argumentar plan nacional con inicio en la Región Metropolitana</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>No tener ingresos por ventas (personas jurídicas) y primera venta durante la ejecución</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Bases 3, 4.1 b), 13.3</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Mantener el demo sin cobros reales</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Proyecto</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Objetivo alineado: validación técnica y comercial (no compra de equipos ni consultorías)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Bases 2.1</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Redactar el plan de validación</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Al menos 2 personas (hasta 3 cofundadores) con roles complementarios</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.2, 9.2</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Confirmar roles y perfil comercial</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Dedicación horaria comprometida (máx. 40 a 44 h semanales) y verificable</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Bases 8 d)</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Completar horas por persona</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Participantes</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Entidad Patrocinadora de la nómina de Semilla Inicia habilitada para la región</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.3</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Buscar y elegir; preguntar a INACAP</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Participantes</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Mentoría de una red reconocida por Corfo, iniciada en los primeros 4 meses</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Bases 3, 7.1</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Elegir la red con la patrocinadora</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Formulario</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>a) Solución: problema, valor agregado, estado de desarrollo, ODS</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Bases 8 a)</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Completar docs/corfo/BORRADOR_POSTULACION.md</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Formulario</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>b) Escalabilidad: modelo de negocios, clientes, competencia, mercado, región</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Bases 8 b)</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Falta mercado y competencia chilena</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Formulario</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>c) Plan de validación con actividades y resultados</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Bases 8 c)</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Ajustar con fechas reales (hoja Gantt)</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Formulario</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>d) Capacidades del equipo y dedicación</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Bases 8 d)</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Completar con datos reales</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Formulario</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>e) Video de máximo 40 s, accesible y con fecha de carga</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Bases 8 e)</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Grabar con el guion del borrador</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Formulario</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Anexo 2 (ODS) y Anexo 3 (estrategia de operación sostenible)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Bases anexos 2 y 3</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Leer los anexos y completar</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Aporte propio de al menos 25 % del costo total</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Bases 6.3</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Completar la hoja Presupuesto</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Subsidio de hasta 75 % con tope de $15.000.000; gastos de inversión hasta 20 % del subsidio; honorarios de socios hasta $700.000 al mes (máx. 2)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Bases 6.1, 12</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Armar el presupuesto dentro de los topes</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Presupuesto</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Incluir la constitución de la sociedad e inicio de actividades (actividad obligatoria si es persona natural)</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Bases 7.1 b)</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Cotizar abogado y notaría</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Después de aprobar</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Contrato con la Entidad Patrocinadora y antecedentes de edad y residencia (15 días)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Bases 13.3, Anexo 1</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Futuro</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Después de aprobar</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Constituir la persona jurídica: beneficiario con participación mayoritaria; cada integrante con al menos 5 %</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Bases 4.4.2</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Futuro</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Acordar el reparto desde ya</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Fuente: bases técnicas de Semilla Inicia (Res. Exenta 1498/2025) y ficha oficial del concurso Biobío 2026. Cada convocatoria puede cambiar los requisitos: leer las bases del llamado exacto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Cumple</t>
+        </is>
+      </c>
+      <c r="D29" s="10">
+        <f>COUNTIF(E2:E25,"Cumple")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Por verificar</t>
+        </is>
+      </c>
+      <c r="D30" s="10">
+        <f>COUNTIF(E2:E25,"Por verificar")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Borrador</t>
+        </is>
+      </c>
+      <c r="D31" s="10">
+        <f>COUNTIF(E2:E25,"Borrador")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="D32" s="10">
+        <f>COUNTIF(E2:E25,"Falta")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Futuro</t>
+        </is>
+      </c>
+      <c r="D33" s="10">
+        <f>COUNTIF(E2:E25,"Futuro")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G25"/>
+  <conditionalFormatting sqref="A2:G200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$E2="Cumple"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>$E2="Borrador"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>$E2="Por verificar"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$E2="Falta"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Cumple,Por verificar,Borrador,Falta,Futuro"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Inicio (mes)</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Fin (mes)</t>
+        </is>
+      </c>
+      <c r="E1" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H1" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I1" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="J1" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="K1" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="L1" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="M1" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="N1" s="23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Constituir la sociedad e iniciar actividades en el SII</t>
+        </is>
+      </c>
+      <c r="B2" s="25" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="C2" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="26" t="n"/>
+      <c r="F2" s="26" t="n"/>
+      <c r="G2" s="26" t="n"/>
+      <c r="H2" s="26" t="n"/>
+      <c r="I2" s="26" t="n"/>
+      <c r="J2" s="26" t="n"/>
+      <c r="K2" s="26" t="n"/>
+      <c r="L2" s="26" t="n"/>
+      <c r="M2" s="26" t="n"/>
+      <c r="N2" s="26" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Firmar el contrato con la Entidad Patrocinadora</t>
+        </is>
+      </c>
+      <c r="B3" s="25" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="26" t="n"/>
+      <c r="F3" s="26" t="n"/>
+      <c r="G3" s="26" t="n"/>
+      <c r="H3" s="26" t="n"/>
+      <c r="I3" s="26" t="n"/>
+      <c r="J3" s="26" t="n"/>
+      <c r="K3" s="26" t="n"/>
+      <c r="L3" s="26" t="n"/>
+      <c r="M3" s="26" t="n"/>
+      <c r="N3" s="26" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Definir el modelo de negocios con la mentoría</t>
+        </is>
+      </c>
+      <c r="B4" s="25" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="26" t="n"/>
+      <c r="F4" s="26" t="n"/>
+      <c r="G4" s="26" t="n"/>
+      <c r="H4" s="26" t="n"/>
+      <c r="I4" s="26" t="n"/>
+      <c r="J4" s="26" t="n"/>
+      <c r="K4" s="26" t="n"/>
+      <c r="L4" s="26" t="n"/>
+      <c r="M4" s="26" t="n"/>
+      <c r="N4" s="26" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Producción técnica: pasarela real, correo transaccional, T&amp;C, claves</t>
+        </is>
+      </c>
+      <c r="B5" s="25" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
+      <c r="H5" s="26" t="n"/>
+      <c r="I5" s="26" t="n"/>
+      <c r="J5" s="26" t="n"/>
+      <c r="K5" s="26" t="n"/>
+      <c r="L5" s="26" t="n"/>
+      <c r="M5" s="26" t="n"/>
+      <c r="N5" s="26" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Cumplimiento Ley 21.719 y revisión legal</t>
+        </is>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="26" t="n"/>
+      <c r="F6" s="26" t="n"/>
+      <c r="G6" s="26" t="n"/>
+      <c r="H6" s="26" t="n"/>
+      <c r="I6" s="26" t="n"/>
+      <c r="J6" s="26" t="n"/>
+      <c r="K6" s="26" t="n"/>
+      <c r="L6" s="26" t="n"/>
+      <c r="M6" s="26" t="n"/>
+      <c r="N6" s="26" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Mentoría (debe iniciar antes del mes 4)</t>
+        </is>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="26" t="n"/>
+      <c r="G7" s="26" t="n"/>
+      <c r="H7" s="26" t="n"/>
+      <c r="I7" s="26" t="n"/>
+      <c r="J7" s="26" t="n"/>
+      <c r="K7" s="26" t="n"/>
+      <c r="L7" s="26" t="n"/>
+      <c r="M7" s="26" t="n"/>
+      <c r="N7" s="26" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Estrategia de operación sostenible (Anexo 3)</t>
+        </is>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="26" t="n"/>
+      <c r="F8" s="26" t="n"/>
+      <c r="G8" s="26" t="n"/>
+      <c r="H8" s="26" t="n"/>
+      <c r="I8" s="26" t="n"/>
+      <c r="J8" s="26" t="n"/>
+      <c r="K8" s="26" t="n"/>
+      <c r="L8" s="26" t="n"/>
+      <c r="M8" s="26" t="n"/>
+      <c r="N8" s="26" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Piloto con proveedores y clientes reales; validación comercial</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="26" t="n"/>
+      <c r="F9" s="26" t="n"/>
+      <c r="G9" s="26" t="n"/>
+      <c r="H9" s="26" t="n"/>
+      <c r="I9" s="26" t="n"/>
+      <c r="J9" s="26" t="n"/>
+      <c r="K9" s="26" t="n"/>
+      <c r="L9" s="26" t="n"/>
+      <c r="M9" s="26" t="n"/>
+      <c r="N9" s="26" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Primera venta: servicio pagado en la plataforma</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="E10" s="26" t="n"/>
+      <c r="F10" s="26" t="n"/>
+      <c r="G10" s="26" t="n"/>
+      <c r="H10" s="26" t="n"/>
+      <c r="I10" s="26" t="n"/>
+      <c r="J10" s="26" t="n"/>
+      <c r="K10" s="26" t="n"/>
+      <c r="L10" s="26" t="n"/>
+      <c r="M10" s="26" t="n"/>
+      <c r="N10" s="26" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Medición, ajustes y plan de escalamiento a otras regiones</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" s="26" t="n"/>
+      <c r="F11" s="26" t="n"/>
+      <c r="G11" s="26" t="n"/>
+      <c r="H11" s="26" t="n"/>
+      <c r="I11" s="26" t="n"/>
+      <c r="J11" s="26" t="n"/>
+      <c r="K11" s="26" t="n"/>
+      <c r="L11" s="26" t="n"/>
+      <c r="M11" s="26" t="n"/>
+      <c r="N11" s="26" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>Informe final y rendición</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="26" t="n"/>
+      <c r="F12" s="26" t="n"/>
+      <c r="G12" s="26" t="n"/>
+      <c r="H12" s="26" t="n"/>
+      <c r="I12" s="26" t="n"/>
+      <c r="J12" s="26" t="n"/>
+      <c r="K12" s="26" t="n"/>
+      <c r="L12" s="26" t="n"/>
+      <c r="M12" s="26" t="n"/>
+      <c r="N12" s="26" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Meses de ejecución desde la firma del convenio (máximo 10, más 2 de prórroga excepcional). Cambia el inicio y el fin (azul) y la barra se mueve sola. Cuando se conozca la fecha de apertura, pasa estas actividades a Planner con fechas reales.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E2:N32">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>AND($C2&lt;&gt;"",E$1&gt;=$C2,E$1&lt;=$D2)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3099,12 +4499,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Corfo</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Corregir hallazgos de la revisión externa (Webpay doble confirmación, sesiones, cancelar/rechazar, eliminación con espera de 15 días, expiración de solicitudes)</t>
+          <t>Elegir al beneficiario (persona natural) y acordar el reparto de la futura sociedad entre los tres antes de postular</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -3114,24 +4514,24 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Dueño</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr"/>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr"/>
+      <c r="H36" s="6" t="inlineStr"/>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Si se aprueba hay que constituir la sociedad: el beneficiario debe tener participación mayoritaria y cada integrante al menos 5 %</t>
+        </is>
+      </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>plan-ajustes.md</t>
+          <t>docs/corfo/README.md</t>
         </is>
       </c>
     </row>
@@ -3143,12 +4543,12 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Corfo</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Invalidar access tokens al cambiar la clave o eliminar la cuenta; cerrar sesión en todos los dispositivos con código por correo</t>
+          <t>Buscar la Entidad Patrocinadora (nómina de Semilla Inicia de la región) y la red de mentores; preguntar a INACAP</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -3158,24 +4558,24 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Dueño</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr"/>
-      <c r="H37" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="I37" s="5" t="inlineStr"/>
+      <c r="H37" s="6" t="inlineStr"/>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Ambas son obligatorias en las bases</t>
+        </is>
+      </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+          <t>docs/corfo/README.md</t>
         </is>
       </c>
     </row>
@@ -3187,12 +4587,12 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Corfo</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Flow y Mercado Pago como medios de pago (código, probado con mocks)</t>
+          <t>Estudio de competencia chilena y tamaño de mercado con fuentes citables (la tesis solo compara con plataformas extranjeras)</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -3202,28 +4602,24 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Dueño</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr"/>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
+      <c r="H38" s="6" t="inlineStr"/>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Falta probar en sandbox real</t>
+          <t>Pesa en Innovación (40 %) y Escalabilidad (30 %)</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+          <t>docs/corfo/DE_LA_TESIS_A_LA_POSTULACION.md</t>
         </is>
       </c>
     </row>
@@ -3235,39 +4631,39 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Corfo</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Registro de reembolsos, más avisos por correo, chequeos de claves inseguras</t>
+          <t>Completar el borrador de postulación: equipo, horas, ODS, sostenibilidad, metas de piloto</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Dueño</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="I39" s="5" t="inlineStr"/>
+      <c r="H39" s="6" t="inlineStr"/>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Claude puede ayudar a redactar con tus datos</t>
+        </is>
+      </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+          <t>docs/corfo/BORRADOR_POSTULACION.md</t>
         </is>
       </c>
     </row>
@@ -3279,12 +4675,12 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Corfo</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Comisión por tramos que paga el cliente encima del precio + análisis de costos de pasarelas</t>
+          <t>Grabar el video de máximo 40 segundos (alojado con fecha de carga) y probar que abre sin clave</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -3294,24 +4690,24 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Hecho</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Dueño</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr"/>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="I40" s="5" t="inlineStr"/>
+      <c r="H40" s="6" t="inlineStr"/>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Si no abre, la postulación no se evalúa</t>
+        </is>
+      </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>ANALISIS_COMISION.md</t>
+          <t>docs/corfo/BORRADOR_POSTULACION.md</t>
         </is>
       </c>
     </row>
@@ -3323,45 +4719,629 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
+          <t>Corfo</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Vigilar la apertura de la próxima convocatoria de Semilla Inicia y leer las bases exactas de ese llamado</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr"/>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Las de 2026 ya cerraron; no hay una abierta hoy</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>docs/corfo/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>T-041</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Corfo</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>No cobrar dinero real ni constituir la sociedad antes de saber el resultado</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="inlineStr"/>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Persona jurídica sin ventas; la primera venta es parte de la ejecución</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>docs/corfo/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>T-042</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Ley 21.719 (vigencia 1-dic-2026): ejecutar el plan de adecuación semana a semana</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Abogado</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>2026-12-01</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr">
+        <is>
+          <t>Ver preguntas para el abogado en el plan</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>docs/cumplimiento/PLAN_ADECUACION_LEY_21719.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>T-043</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Contratos o DPA con los encargados y decisión sobre transferencias internacionales (EE. UU., Brasil)</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>Abogado</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr"/>
+      <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>docs/cumplimiento/PLAN_ADECUACION_LEY_21719.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>T-044</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Simulacro de brecha de seguridad y de solicitud de derechos; designar suplente</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>docs/legal/protocolo-de-brechas.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>T-045</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Actualizar la EIPD y el registro de tratamientos con el video de verificación, Flow, Mercado Pago y los avisos por correo</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr"/>
+      <c r="H46" s="6" t="inlineStr"/>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>docs/cumplimiento/PLAN_ADECUACION_LEY_21719.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>T-046</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Desarrollo</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Armar la carta Gantt definitiva en Planner con fechas reales cuando se conozca la apertura</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Convocatoria abierta</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr"/>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>Hoja Gantt del Excel como base</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>hoja Gantt</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>T-047</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
           <t>Hecho</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Corregir hallazgos de la revisión externa (Webpay doble confirmación, sesiones, cancelar/rechazar, eliminación con espera de 15 días, expiración de solicitudes)</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G48" s="6" t="inlineStr"/>
+      <c r="H48" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>plan-ajustes.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>T-048</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Invalidar access tokens al cambiar la clave o eliminar la cuenta; cerrar sesión en todos los dispositivos con código por correo</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>T-049</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Flow y Mercado Pago como medios de pago (código, probado con mocks)</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr"/>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Falta probar en sandbox real</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>T-050</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Registro de reembolsos, más avisos por correo, chequeos de claves inseguras</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr"/>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>T-051</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Comisión por tramos que paga el cliente encima del precio + análisis de costos de pasarelas</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr"/>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>ANALISIS_COMISION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>T-052</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Guía de postulación a Corfo con las bases oficiales (Semilla Inicia), borrador de postulación y puente tesis → postulación; plan de adecuación a la Ley 21.719</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr"/>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr">
+        <is>
+          <t>Borradores a completar con tus datos</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>docs/corfo/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>T-053</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>Verificación sin biometría con video + cédula revisada por un moderador (el video se borra al resolver)</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>Hecho</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr"/>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr"/>
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr"/>
-      <c r="J41" s="5" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr">
         <is>
           <t>docs/adr/0006</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J41"/>
-  <conditionalFormatting sqref="A2:J141">
+  <autoFilter ref="A1:J54"/>
+  <conditionalFormatting sqref="A2:J154">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$E2="Hecho"</formula>
     </cfRule>
@@ -3373,13 +5353,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="D2:D141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Alta,Media,Baja"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,En curso,Bloqueado,Hecho"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F141" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Dueño,Claude,Tercero"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3393,7 +5373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -4642,10 +6622,400 @@
         <v/>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="5">
+        <f>Tareas!C42</f>
+        <v/>
+      </c>
+      <c r="B42" s="5">
+        <f>Tareas!B42</f>
+        <v/>
+      </c>
+      <c r="C42" s="5">
+        <f>IF(Tareas!E42="Hecho","Completada",IF(Tareas!E42="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D42" s="5">
+        <f>IF(Tareas!D42="Alta","Importante",IF(Tareas!D42="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E42" s="5">
+        <f>IF(Tareas!H42="","",Tareas!H42)</f>
+        <v/>
+      </c>
+      <c r="F42" s="5">
+        <f>Tareas!F42</f>
+        <v/>
+      </c>
+      <c r="G42" s="5">
+        <f>Tareas!I42</f>
+        <v/>
+      </c>
+    </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>Se llena sola desde la hoja Tareas (filas 2 a 41). Si agregas tareas, copia las fórmulas hacia abajo.</t>
+      <c r="A43" s="5">
+        <f>Tareas!C43</f>
+        <v/>
+      </c>
+      <c r="B43" s="5">
+        <f>Tareas!B43</f>
+        <v/>
+      </c>
+      <c r="C43" s="5">
+        <f>IF(Tareas!E43="Hecho","Completada",IF(Tareas!E43="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D43" s="5">
+        <f>IF(Tareas!D43="Alta","Importante",IF(Tareas!D43="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E43" s="5">
+        <f>IF(Tareas!H43="","",Tareas!H43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="5">
+        <f>Tareas!F43</f>
+        <v/>
+      </c>
+      <c r="G43" s="5">
+        <f>Tareas!I43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5">
+        <f>Tareas!C44</f>
+        <v/>
+      </c>
+      <c r="B44" s="5">
+        <f>Tareas!B44</f>
+        <v/>
+      </c>
+      <c r="C44" s="5">
+        <f>IF(Tareas!E44="Hecho","Completada",IF(Tareas!E44="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D44" s="5">
+        <f>IF(Tareas!D44="Alta","Importante",IF(Tareas!D44="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E44" s="5">
+        <f>IF(Tareas!H44="","",Tareas!H44)</f>
+        <v/>
+      </c>
+      <c r="F44" s="5">
+        <f>Tareas!F44</f>
+        <v/>
+      </c>
+      <c r="G44" s="5">
+        <f>Tareas!I44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5">
+        <f>Tareas!C45</f>
+        <v/>
+      </c>
+      <c r="B45" s="5">
+        <f>Tareas!B45</f>
+        <v/>
+      </c>
+      <c r="C45" s="5">
+        <f>IF(Tareas!E45="Hecho","Completada",IF(Tareas!E45="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D45" s="5">
+        <f>IF(Tareas!D45="Alta","Importante",IF(Tareas!D45="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E45" s="5">
+        <f>IF(Tareas!H45="","",Tareas!H45)</f>
+        <v/>
+      </c>
+      <c r="F45" s="5">
+        <f>Tareas!F45</f>
+        <v/>
+      </c>
+      <c r="G45" s="5">
+        <f>Tareas!I45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5">
+        <f>Tareas!C46</f>
+        <v/>
+      </c>
+      <c r="B46" s="5">
+        <f>Tareas!B46</f>
+        <v/>
+      </c>
+      <c r="C46" s="5">
+        <f>IF(Tareas!E46="Hecho","Completada",IF(Tareas!E46="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D46" s="5">
+        <f>IF(Tareas!D46="Alta","Importante",IF(Tareas!D46="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E46" s="5">
+        <f>IF(Tareas!H46="","",Tareas!H46)</f>
+        <v/>
+      </c>
+      <c r="F46" s="5">
+        <f>Tareas!F46</f>
+        <v/>
+      </c>
+      <c r="G46" s="5">
+        <f>Tareas!I46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5">
+        <f>Tareas!C47</f>
+        <v/>
+      </c>
+      <c r="B47" s="5">
+        <f>Tareas!B47</f>
+        <v/>
+      </c>
+      <c r="C47" s="5">
+        <f>IF(Tareas!E47="Hecho","Completada",IF(Tareas!E47="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D47" s="5">
+        <f>IF(Tareas!D47="Alta","Importante",IF(Tareas!D47="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E47" s="5">
+        <f>IF(Tareas!H47="","",Tareas!H47)</f>
+        <v/>
+      </c>
+      <c r="F47" s="5">
+        <f>Tareas!F47</f>
+        <v/>
+      </c>
+      <c r="G47" s="5">
+        <f>Tareas!I47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5">
+        <f>Tareas!C48</f>
+        <v/>
+      </c>
+      <c r="B48" s="5">
+        <f>Tareas!B48</f>
+        <v/>
+      </c>
+      <c r="C48" s="5">
+        <f>IF(Tareas!E48="Hecho","Completada",IF(Tareas!E48="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D48" s="5">
+        <f>IF(Tareas!D48="Alta","Importante",IF(Tareas!D48="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E48" s="5">
+        <f>IF(Tareas!H48="","",Tareas!H48)</f>
+        <v/>
+      </c>
+      <c r="F48" s="5">
+        <f>Tareas!F48</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>Tareas!I48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5">
+        <f>Tareas!C49</f>
+        <v/>
+      </c>
+      <c r="B49" s="5">
+        <f>Tareas!B49</f>
+        <v/>
+      </c>
+      <c r="C49" s="5">
+        <f>IF(Tareas!E49="Hecho","Completada",IF(Tareas!E49="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D49" s="5">
+        <f>IF(Tareas!D49="Alta","Importante",IF(Tareas!D49="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E49" s="5">
+        <f>IF(Tareas!H49="","",Tareas!H49)</f>
+        <v/>
+      </c>
+      <c r="F49" s="5">
+        <f>Tareas!F49</f>
+        <v/>
+      </c>
+      <c r="G49" s="5">
+        <f>Tareas!I49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5">
+        <f>Tareas!C50</f>
+        <v/>
+      </c>
+      <c r="B50" s="5">
+        <f>Tareas!B50</f>
+        <v/>
+      </c>
+      <c r="C50" s="5">
+        <f>IF(Tareas!E50="Hecho","Completada",IF(Tareas!E50="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D50" s="5">
+        <f>IF(Tareas!D50="Alta","Importante",IF(Tareas!D50="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E50" s="5">
+        <f>IF(Tareas!H50="","",Tareas!H50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="5">
+        <f>Tareas!F50</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>Tareas!I50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5">
+        <f>Tareas!C51</f>
+        <v/>
+      </c>
+      <c r="B51" s="5">
+        <f>Tareas!B51</f>
+        <v/>
+      </c>
+      <c r="C51" s="5">
+        <f>IF(Tareas!E51="Hecho","Completada",IF(Tareas!E51="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D51" s="5">
+        <f>IF(Tareas!D51="Alta","Importante",IF(Tareas!D51="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E51" s="5">
+        <f>IF(Tareas!H51="","",Tareas!H51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="5">
+        <f>Tareas!F51</f>
+        <v/>
+      </c>
+      <c r="G51" s="5">
+        <f>Tareas!I51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5">
+        <f>Tareas!C52</f>
+        <v/>
+      </c>
+      <c r="B52" s="5">
+        <f>Tareas!B52</f>
+        <v/>
+      </c>
+      <c r="C52" s="5">
+        <f>IF(Tareas!E52="Hecho","Completada",IF(Tareas!E52="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D52" s="5">
+        <f>IF(Tareas!D52="Alta","Importante",IF(Tareas!D52="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E52" s="5">
+        <f>IF(Tareas!H52="","",Tareas!H52)</f>
+        <v/>
+      </c>
+      <c r="F52" s="5">
+        <f>Tareas!F52</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>Tareas!I52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5">
+        <f>Tareas!C53</f>
+        <v/>
+      </c>
+      <c r="B53" s="5">
+        <f>Tareas!B53</f>
+        <v/>
+      </c>
+      <c r="C53" s="5">
+        <f>IF(Tareas!E53="Hecho","Completada",IF(Tareas!E53="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D53" s="5">
+        <f>IF(Tareas!D53="Alta","Importante",IF(Tareas!D53="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E53" s="5">
+        <f>IF(Tareas!H53="","",Tareas!H53)</f>
+        <v/>
+      </c>
+      <c r="F53" s="5">
+        <f>Tareas!F53</f>
+        <v/>
+      </c>
+      <c r="G53" s="5">
+        <f>Tareas!I53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5">
+        <f>Tareas!C54</f>
+        <v/>
+      </c>
+      <c r="B54" s="5">
+        <f>Tareas!B54</f>
+        <v/>
+      </c>
+      <c r="C54" s="5">
+        <f>IF(Tareas!E54="Hecho","Completada",IF(Tareas!E54="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D54" s="5">
+        <f>IF(Tareas!D54="Alta","Importante",IF(Tareas!D54="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E54" s="5">
+        <f>IF(Tareas!H54="","",Tareas!H54)</f>
+        <v/>
+      </c>
+      <c r="F54" s="5">
+        <f>Tareas!F54</f>
+        <v/>
+      </c>
+      <c r="G54" s="5">
+        <f>Tareas!I54</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>Se llena sola desde la hoja Tareas (filas 2 a 54). Si agregas tareas, copia las fórmulas hacia abajo.</t>
         </is>
       </c>
     </row>
@@ -4660,7 +7030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5755,15 +8125,38 @@
       </c>
       <c r="E47" s="5" t="inlineStr"/>
     </row>
-    <row r="49">
-      <c r="A49" s="8" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>c687bee</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Pagos</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Agrega comisión por tramos, verificación con video y tablero de seguimiento</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>Cada fila es un commit de master (git log). Para ver el detalle: git show &lt;commit&gt;. Agrega notas a mano si hace falta.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E47"/>
+  <autoFilter ref="A1:E48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Registra en el seguimiento las decisiones de estrategia y las tareas de los bloques 1 a 4
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -2928,7 +2928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5336,6 +5336,182 @@
       <c r="J54" s="5" t="inlineStr">
         <is>
           <t>docs/adr/0006</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>T-054</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 1: medición de impacto (situación laboral, tipo de servicio, reparación evitó reemplazo, reporte_impacto)</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="6" t="n"/>
+      <c r="I55" s="5" t="inlineStr">
+        <is>
+          <t>Agregados con supresión de grupos &lt; 5; finalidad en política y registro de actividades</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>Prompt de implementación Corfo 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>T-055</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 2: calculadora gratuita de valorización (/calculadora, PDF/xlsx, plantillas, ItemPresupuesto extendido)</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Pública sin cuenta; contador de uso anónimo</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr">
+        <is>
+          <t>Prompt de implementación Corfo 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>T-056</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 3: boleta fase 1 (folio de boleta de honorarios, primera boleta)</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="6" t="n"/>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Sin integración con el SII; KeyServ no emite boletas</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>Prompt de implementación Corfo 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>T-057</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 4: vía sin historial (destacar cédula + video en registro y portada)</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Copy honesto según ADR 0006</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>Prompt de implementación Corfo 2026-10-23</t>
         </is>
       </c>
     </row>
@@ -5373,7 +5549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -7012,10 +7188,130 @@
         <v/>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="5">
+        <f>Tareas!C55</f>
+        <v/>
+      </c>
+      <c r="B55" s="5">
+        <f>Tareas!B55</f>
+        <v/>
+      </c>
+      <c r="C55" s="5">
+        <f>IF(Tareas!E55="Hecho","Completada",IF(Tareas!E55="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D55" s="5">
+        <f>IF(Tareas!D55="Alta","Importante",IF(Tareas!D55="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E55" s="5">
+        <f>IF(Tareas!H55="","",Tareas!H55)</f>
+        <v/>
+      </c>
+      <c r="F55" s="5">
+        <f>Tareas!F55</f>
+        <v/>
+      </c>
+      <c r="G55" s="5">
+        <f>Tareas!I55</f>
+        <v/>
+      </c>
+    </row>
     <row r="56">
-      <c r="A56" s="8" t="inlineStr">
-        <is>
-          <t>Se llena sola desde la hoja Tareas (filas 2 a 54). Si agregas tareas, copia las fórmulas hacia abajo.</t>
+      <c r="A56" s="5">
+        <f>Tareas!C56</f>
+        <v/>
+      </c>
+      <c r="B56" s="5">
+        <f>Tareas!B56</f>
+        <v/>
+      </c>
+      <c r="C56" s="5">
+        <f>IF(Tareas!E56="Hecho","Completada",IF(Tareas!E56="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D56" s="5">
+        <f>IF(Tareas!D56="Alta","Importante",IF(Tareas!D56="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E56" s="5">
+        <f>IF(Tareas!H56="","",Tareas!H56)</f>
+        <v/>
+      </c>
+      <c r="F56" s="5">
+        <f>Tareas!F56</f>
+        <v/>
+      </c>
+      <c r="G56" s="5">
+        <f>Tareas!I56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5">
+        <f>Tareas!C57</f>
+        <v/>
+      </c>
+      <c r="B57" s="5">
+        <f>Tareas!B57</f>
+        <v/>
+      </c>
+      <c r="C57" s="5">
+        <f>IF(Tareas!E57="Hecho","Completada",IF(Tareas!E57="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D57" s="5">
+        <f>IF(Tareas!D57="Alta","Importante",IF(Tareas!D57="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E57" s="5">
+        <f>IF(Tareas!H57="","",Tareas!H57)</f>
+        <v/>
+      </c>
+      <c r="F57" s="5">
+        <f>Tareas!F57</f>
+        <v/>
+      </c>
+      <c r="G57" s="5">
+        <f>Tareas!I57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5">
+        <f>Tareas!C58</f>
+        <v/>
+      </c>
+      <c r="B58" s="5">
+        <f>Tareas!B58</f>
+        <v/>
+      </c>
+      <c r="C58" s="5">
+        <f>IF(Tareas!E58="Hecho","Completada",IF(Tareas!E58="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D58" s="5">
+        <f>IF(Tareas!D58="Alta","Importante",IF(Tareas!D58="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E58" s="5">
+        <f>IF(Tareas!H58="","",Tareas!H58)</f>
+        <v/>
+      </c>
+      <c r="F58" s="5">
+        <f>Tareas!F58</f>
+        <v/>
+      </c>
+      <c r="G58" s="5">
+        <f>Tareas!I58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Se llena sola desde la hoja Tareas (filas 2 a 58). Si agregas tareas, copia las fórmulas hacia abajo.</t>
         </is>
       </c>
     </row>
@@ -8167,7 +8463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8675,6 +8971,166 @@
       <c r="F16" s="5" t="inlineStr">
         <is>
           <t>PLAN_FLUJO_DE_DINERO.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>D-016</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Encuadre de la postulación: inclusión laboral y formalización, no antifraude</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>docs/corfo/RESUMEN_PARA_PLANIFICACION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>D-017</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Economía circular = reparar y mantener en vez de reemplazar; el ingreso que queda en la comuna se reporta aparte como "economía local"</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>docs/corfo/RESUMEN_PARA_PLANIFICACION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>D-018</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Calculadora de valorización gratuita y abierta sin cuenta</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>D-019</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Boleta fase 1: el proveedor emite en sii.cl y KeyServ registra el folio; integración directa con el SII queda para después</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>D-020</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>ODS declarados: 8 (principal), 10 y 12. No se declaran el 5 ni el 16</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>docs/corfo/BORRADOR_POSTULACION.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega medición de impacto: preguntas voluntarias, tipo de servicio y reporte agregado
Situación laboral previa y género (voluntarios, en registro y Preferencias),
tipo de servicio por publicación, pregunta de reemplazo al calificar una
reparación y manage.py reporte_impacto, que solo entrega agregados y oculta
grupos de menos de 5 personas. ADR 0008 y migración 0044.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -5362,7 +5362,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -5371,10 +5371,14 @@
         </is>
       </c>
       <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Agregados con supresión de grupos &lt; 5; finalidad en política y registro de actividades</t>
+          <t>Migración 0044; ADR 0008; reporte_impacto; falta revisión legal de la finalidad (Pendientes_dueño)</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
@@ -8463,7 +8467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9131,6 +9135,38 @@
       <c r="F21" s="5" t="inlineStr">
         <is>
           <t>docs/corfo/BORRADOR_POSTULACION.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>D-021</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Medición de impacto: datos voluntarios (situación laboral previa, género), tipo de servicio y pregunta de reemplazo; reporte solo agregado con supresión de grupos &lt; 5 y sin cuentas demo</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Claude (técnica) / Dueño (estrategia)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>docs/adr/0008</t>
         </is>
       </c>
     </row>
@@ -9151,7 +9187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9470,6 +9506,29 @@
       </c>
       <c r="D14" s="6" t="inlineStr"/>
       <c r="E14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Abogado: medición de impacto</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Revisar la finalidad escrita en el registro y en la política, la base de licitud (consentimiento voluntario y revocable), si situación laboral previa y género son dato sensible bajo la Ley 21.719 y el plazo de conservación</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>ADR 0008; registro-actividades-tratamiento.md</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E14"/>

</xml_diff>

<commit_message>
Agrega la calculadora gratuita de valorización con boleta de honorarios
Ruta publica /calculadora (sin cuenta): materiales, traslado, mano de obra,
herramientas, imprevistos y ganancia; con boleta calcula el precio para que
tras la retencion quede lo deseado y suma la comision real. Exporta PDF y
planilla xlsx con formulas editables. Con cuenta guarda plantillas que se
cargan en la hoja de presupuesto al confirmar. ItemPresupuesto gana detalle
opcional (migracion 0045) y hay un contador anonimo de uso para el reporte.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -5410,7 +5410,7 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -5419,10 +5419,14 @@
         </is>
       </c>
       <c r="G56" s="6" t="n"/>
-      <c r="H56" s="6" t="n"/>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Pública sin cuenta; contador de uso anónimo</t>
+          <t>Migración 0045; ADR 0009; falta que un contador confirme la retención (Pendientes_dueño)</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
@@ -8448,6 +8452,33 @@
       </c>
       <c r="E48" s="5" t="inlineStr"/>
     </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>e20bfac</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Agrega medición de impacto: preguntas voluntarias, tipo de servicio y reporte agregado</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 1 (T-054)</t>
+        </is>
+      </c>
+    </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
@@ -8467,7 +8498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9167,6 +9198,38 @@
       <c r="F22" s="5" t="inlineStr">
         <is>
           <t>docs/adr/0008</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>D-022</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Calculadora de valorización: el cálculo vive en el servidor (usa la comisión real), pesos enteros con boleta redondeada hacia arriba, exportación PDF/xlsx en el servidor, plantillas por cuenta, hoja de presupuesto extendida, contador anónimo con hash mensual</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Claude (técnica) / Dueño (estrategia)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>docs/adr/0009</t>
         </is>
       </c>
     </row>
@@ -9187,7 +9250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9527,6 +9590,52 @@
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>ADR 0008; registro-actividades-tratamiento.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Contador: boleta de honorarios en la calculadora</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Confirmar la retención vigente (la calculadora usa 16 % para 2027, editable con CALCULADORA_RETENCION_BOLETA) y cómo van los materiales dentro de una boleta de honorarios</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>ADR 0009</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Abogado: contador anónimo de la calculadora</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Confirmar si el identificador aleatorio del navegador (hash mensual, sin IP ni cuenta) cuenta como dato personal y si basta con lo declarado en la política</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>ADR 0009; registro-actividades-tratamiento.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega el registro del folio de la boleta de honorarios (fase 1, sin SII)
El proveedor emite su boleta en sii.cl y registra aqui el folio de un trabajo
pagado; el cliente lo ve para revisarlo. KeyServ no emite boletas ni verifica
el folio. reporte_impacto cuenta servicios con boleta y primeras boletas.
ADR 0010 y migracion 0046.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -5458,7 +5458,7 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -5467,10 +5467,14 @@
         </is>
       </c>
       <c r="G57" s="6" t="n"/>
-      <c r="H57" s="6" t="n"/>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Sin integración con el SII; KeyServ no emite boletas</t>
+          <t>Migración 0046; ADR 0010; el folio es declarado, no verificado con el SII</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
@@ -8480,9 +8484,29 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
-        <is>
-          <t>Cada fila es un commit de master (git log). Para ver el detalle: git show &lt;commit&gt;. Agrega notas a mano si hace falta.</t>
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>b525d74</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Agrega la calculadora gratuita de valorización con boleta de honorarios</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 2 (T-055)</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9230,6 +9254,38 @@
       <c r="F23" s="5" t="inlineStr">
         <is>
           <t>docs/adr/0009</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>D-023</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Boleta fase 1: el proveedor registra el folio de un trabajo pagado (uno por contratación, no repetido por proveedor, una sola primera boleta); KeyServ no emite ni verifica; el folio se conserva al anonimizar la cuenta</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Claude (técnica) / Dueño (estrategia)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>docs/adr/0010</t>
         </is>
       </c>
     </row>
@@ -9250,7 +9306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9636,6 +9692,29 @@
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>ADR 0009; registro-actividades-tratamiento.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Contador/abogado: boleta fase 2</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Antes de verificar el folio con el SII o emitir boletas desde KeyServ: tratamiento tributario de la comisión, si hace falta ser emisor autorizado y qué integración corresponde</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>ADR 0010; PLAN_FLUJO_DE_DINERO.md §4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Destaca la vía sin historial (cédula y video) y corrige el aviso de fotos del rostro
La portada y el registro explican que quien nunca ha trabajado con boleta puede
empezar verificando su identidad con la cédula y un video que revisa una
persona, sin prometer una consulta al Registro Civil. El aviso de privacidad
de la portada ya no dice que no se guardan fotos del rostro. Actualiza
CLAUDE.md y el seguimiento.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -2075,7 +2075,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Completar docs/corfo/BORRADOR_POSTULACION.md</t>
+          <t>Reescribir con el encuadre de inclusión laboral y citar cifras reales de manage.py reporte_impacto (docs/corfo/README.md §6); completar docs/corfo/BORRADOR_POSTULACION.md</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -5506,7 +5506,7 @@
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F58" s="6" t="inlineStr">
@@ -5515,10 +5515,14 @@
         </is>
       </c>
       <c r="G58" s="6" t="n"/>
-      <c r="H58" s="6" t="n"/>
+      <c r="H58" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Copy honesto según ADR 0006</t>
+          <t>Solo copy y presentación; se corrigió el aviso "0 fotos de tu rostro guardadas"; sigue pendiente la revisión legal del video y el documento</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
@@ -7338,7 +7342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8507,6 +8511,33 @@
       <c r="E50" s="5" t="inlineStr">
         <is>
           <t>Bloque 2 (T-055)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>32e5bea</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Agrega el registro del folio de la boleta de honorarios (fase 1, sin SII)</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 3 (T-056)</t>
         </is>
       </c>
     </row>
@@ -8522,7 +8553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9286,6 +9317,38 @@
       <c r="F24" s="5" t="inlineStr">
         <is>
           <t>docs/adr/0010</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>D-024</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Vía sin historial: destacar la cédula + video en portada y registro, diciendo que es una revisión humana (no una consulta al Registro Civil); corregir el aviso "0 fotos de tu rostro guardadas"</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Claude (copy) / Dueño (estrategia)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>docs/adr/0006 (actualización 2026-10-23)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Registra en el seguimiento el commit del bloque 4
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -7342,7 +7342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8538,6 +8538,33 @@
       <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Bloque 3 (T-056)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>611ed94</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Código</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Destaca la vía sin historial (cédula y video) y corrige el aviso de fotos del rostro</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Bloque 4 (T-057)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mejora la calculadora: modo normal, confirmar por la calculadora, IVA y reparto del cobro
- Dos modos: Normal (precio simple) y Calculadora de costos.
- Reparto del cobro explicado (comision por tramos, total del cliente, lo que
  recibe el proveedor) y agradecimiento en la pantalla de quien contrata.
- Confirmar contratacion lleva a /calculadora?contratacion=<id> con el precio
  de la publicacion en grande; la contratacion expone publicacion_precio.
- Imprevistos y ganancia opcionales, con explicacion; documento con IVA
  opcional y la retencion explicada como adelanto del impuesto a la renta.
- Registra en el plan la calculadora guiada (T-058).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -2928,7 +2928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J58"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5528,6 +5528,50 @@
       <c r="J58" s="5" t="inlineStr">
         <is>
           <t>Prompt de implementación Corfo 2026-10-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>T-058</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Calculadora guiada: asistente paso a paso con un pequeño guía de indicaciones (guion fijo, sin IA) y resultado simple con «Ver el detalle»</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="6" t="n"/>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>Plan acordado 2026-10-23; ver ESTADO_Y_PROXIMOS_PASOS.md. Conservar modo Normal, confirmar con ?contratacion, plantillas y exportaciones</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
         </is>
       </c>
     </row>
@@ -5565,7 +5609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -7324,13 +7368,46 @@
         <v/>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="5">
+        <f>Tareas!C59</f>
+        <v/>
+      </c>
+      <c r="B59" s="5">
+        <f>Tareas!B59</f>
+        <v/>
+      </c>
+      <c r="C59" s="5">
+        <f>IF(Tareas!E59="Hecho","Completada",IF(Tareas!E59="En curso","En curso","No iniciada"))</f>
+        <v/>
+      </c>
+      <c r="D59" s="5">
+        <f>IF(Tareas!D59="Alta","Importante",IF(Tareas!D59="Media","Media","Baja"))</f>
+        <v/>
+      </c>
+      <c r="E59" s="5">
+        <f>IF(Tareas!H59="","",Tareas!H59)</f>
+        <v/>
+      </c>
+      <c r="F59" s="5">
+        <f>Tareas!F59</f>
+        <v/>
+      </c>
+      <c r="G59" s="5">
+        <f>Tareas!I59</f>
+        <v/>
+      </c>
+    </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>Se llena sola desde la hoja Tareas (filas 2 a 58). Si agregas tareas, copia las fórmulas hacia abajo.</t>
-        </is>
-      </c>
-    </row>
+          <t>Se llena sola desde la hoja Tareas (filas 2 a 59). Si agregas tareas, copia las fórmulas hacia abajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8580,7 +8657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9376,6 +9453,70 @@
       <c r="F25" s="5" t="inlineStr">
         <is>
           <t>docs/adr/0006 (actualización 2026-10-23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>D-025</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Calculadora: "Confirmar contratación" pasa por la calculadora del trabajo; imprevistos y ganancia opcionales; IVA solo como documento opcional (la boleta de honorarios no lleva IVA); la retención se explica como adelanto del impuesto a la renta</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Aprobada</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>docs/adr/0009</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>D-026</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Calculadora guiada (pendiente de implementar): asistente por pasos con un pequeño guía de guion fijo, sin IA externa, y resultado simple con detalle plegable</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Dueño</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Propuesta</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>docs/ESTADO_Y_PROXIMOS_PASOS.md</t>
         </is>
       </c>
     </row>
@@ -9747,7 +9888,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Confirmar la retención vigente (la calculadora usa 16 % para 2027, editable con CALCULADORA_RETENCION_BOLETA) y cómo van los materiales dentro de una boleta de honorarios</t>
+          <t>Confirmar la retención vigente (16 % para 2027, editable con CALCULADORA_RETENCION_BOLETA), quién la retiene cuando el cliente es una persona natural, cómo van los materiales dentro de una boleta de honorarios y el tratamiento del IVA (opción "documento con IVA", 19 %, CALCULADORA_IVA) incluido el crédito fiscal por materiales comprados con factura</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Registra en docs y seguimiento la calculadora guiada, los headers y la exportación (T-058, T-059)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/seguimiento/KeyServ_Seguimiento.xlsx
+++ b/docs/seguimiento/KeyServ_Seguimiento.xlsx
@@ -2928,7 +2928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5554,7 +5554,7 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
@@ -5563,13 +5563,65 @@
         </is>
       </c>
       <c r="G59" s="6" t="n"/>
-      <c r="H59" s="6" t="n"/>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Plan acordado 2026-10-23; ver ESTADO_Y_PROXIMOS_PASOS.md. Conservar modo Normal, confirmar con ?contratacion, plantillas y exportaciones</t>
+          <t>Hecho: asistente por pasos, guía de guion fijo, ayuda por inactividad, resultado en tres cifras y modo «Ver todo junto». Falta revisar en celular.</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
+        <is>
+          <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>T-059</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Header unificado en 18 páginas y exportación (PDF/xlsx) con logo y hoja de referencia de boleta</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>Hecho</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>La hoja de boleta aclara que no es oficial (KeyServ no emite boletas ni verifica folios).</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr">
         <is>
           <t>ESTADO_Y_PROXIMOS_PASOS.md</t>
         </is>
@@ -5609,7 +5661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
@@ -7405,9 +7457,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>